<commit_message>
Replace CI test fixtures with real Dataset3_v2 samples
tests/input_file/*.fastq.gz previously carried fixed-length, constant-
quality synthetic reads (same deprecated generation style as the
generatefastq.py script removed in the prior commit), unrelated to the
actual published Dataset 3 benchmark.

Swapped in a downsampled (5,000-read) subset of four real Dataset3_v2
samples (healthy_15_25_NOLOI, intermediate_16_31_DOI,
reduced_penetrance_17_37_LOICCA, high_expansion_18_75_NOLOI), covering
the NOLOI/DOI/LOICCA interruption categories. Regenerated
expected_results/ and the manual-correction fixture
(CAG_data_for_recalculating_indices.xlsx) to match; verified STRmie-HD
recovers the exact designed CAG/CCG genotype for all four samples at
this depth. Full regression suite passes (2 passed).
</commit_message>
<xml_diff>
--- a/tests/expected_results/Final_report_expected.xlsx
+++ b/tests/expected_results/Final_report_expected.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,62 +417,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Sample</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Instability_Index</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Expansion_Index</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Allele_Ratio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>LOI_CAA</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>LOI_CCA</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>CAG_repeatsPeak_Allele_1</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>CAG_repeatsPeak_Allele_2</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Max_CAG_observed</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>CCG_allele_1</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>CCG_allele_2</t>
         </is>
@@ -493,41 +481,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>reduced_penetrance_17_38_LOICCA.fastq.gz</t>
+          <t>high_expansion_18_75_NOLOI.fastq.gz</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8.327214400285154</v>
+        <v>-0.3125</v>
       </c>
       <c r="C2" t="n">
-        <v>59.15990453460621</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>1.28</v>
+        <v>0.67</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>4.516129032258064</v>
       </c>
       <c r="F2" t="n">
+        <v>6.451612903225806</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>18</v>
+      </c>
+      <c r="I2" t="n">
         <v>75</v>
       </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>17</v>
-      </c>
-      <c r="I2" t="n">
-        <v>37</v>
-      </c>
       <c r="J2" t="n">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="K2" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="L2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -537,77 +525,77 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9.37997184090109</v>
+        <v>-0.1388888888888889</v>
       </c>
       <c r="C3" t="n">
-        <v>71.30264817150064</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>1.11</v>
+        <v>0.45</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>80</v>
+        <v>80.83333333333333</v>
       </c>
       <c r="H3" t="n">
         <v>16</v>
       </c>
       <c r="I3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J3" t="n">
-        <v>99</v>
+        <v>31</v>
       </c>
       <c r="K3" t="n">
+        <v>7</v>
+      </c>
+      <c r="L3" t="n">
         <v>10</v>
-      </c>
-      <c r="L3" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>full_penetrance_22_48_LOI.fastq.gz</t>
+          <t>reduced_penetrance_17_37_LOICCA.fastq.gz</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5.615384615384617</v>
+        <v>-0.025</v>
       </c>
       <c r="C4" t="n">
-        <v>46.94560669456067</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>1.29</v>
+        <v>0.48</v>
       </c>
       <c r="E4" t="n">
-        <v>72</v>
+        <v>2.173913043478261</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>73.91304347826086</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I4" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="J4" t="n">
-        <v>101</v>
+        <v>37</v>
       </c>
       <c r="K4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -617,19 +605,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9.993377483443707</v>
+        <v>-0.8222222222222223</v>
       </c>
       <c r="C5" t="n">
-        <v>80.53914141414141</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -641,7 +629,7 @@
         <v>25</v>
       </c>
       <c r="J5" t="n">
-        <v>99</v>
+        <v>25</v>
       </c>
       <c r="K5" t="n">
         <v>7</v>

</xml_diff>